<commit_message>
Added commutator, conctruction development
</commit_message>
<xml_diff>
--- a/model/param.xlsx
+++ b/model/param.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zzapa\Desktop\Projekty\elektronika\engine-project\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB5A58CD-6F4F-4879-87B2-D8C4256B1A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B44FD8-6B97-49A7-80CF-CDAD2FCA0469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="100">
   <si>
     <t>stator_out_d</t>
   </si>
@@ -222,6 +222,120 @@
   </si>
   <si>
     <t>shaft_lock_2_shaft_insert_corner_finish</t>
+  </si>
+  <si>
+    <t>commutator_plate_D</t>
+  </si>
+  <si>
+    <t>commutator_plate_d</t>
+  </si>
+  <si>
+    <t>commutator_plastic_h</t>
+  </si>
+  <si>
+    <t>commutator_plate_ang</t>
+  </si>
+  <si>
+    <t>commutator_plate_h</t>
+  </si>
+  <si>
+    <t>commutator_plastic_D</t>
+  </si>
+  <si>
+    <t>commutator_plastic_shaft_d</t>
+  </si>
+  <si>
+    <t>commutator_plastic_insert_cut_deepness</t>
+  </si>
+  <si>
+    <t>commutator_plastic_insert_cut_length</t>
+  </si>
+  <si>
+    <t>commutator_plastic_insert_pos</t>
+  </si>
+  <si>
+    <t>commutator_plate_insert_pos</t>
+  </si>
+  <si>
+    <t>casing_lock_hole_r</t>
+  </si>
+  <si>
+    <t>casing_lock_h</t>
+  </si>
+  <si>
+    <t>casing_stator_fix_r</t>
+  </si>
+  <si>
+    <t>casing_stator_fix_h</t>
+  </si>
+  <si>
+    <t>magnet_ring_insert_part_lengthen</t>
+  </si>
+  <si>
+    <t>casing_sidebar_length</t>
+  </si>
+  <si>
+    <t>casing_sidebar_width</t>
+  </si>
+  <si>
+    <t>casing_vent_hole_length</t>
+  </si>
+  <si>
+    <t>casing_vent_hole_width</t>
+  </si>
+  <si>
+    <t>casing_vent_hole_arc</t>
+  </si>
+  <si>
+    <t>sleeve_in_r</t>
+  </si>
+  <si>
+    <t>sleeve_d</t>
+  </si>
+  <si>
+    <t>sleeve_cup_r</t>
+  </si>
+  <si>
+    <t>sleeve_cup_h</t>
+  </si>
+  <si>
+    <t>sleeve_h</t>
+  </si>
+  <si>
+    <t>casing_head_insert_r</t>
+  </si>
+  <si>
+    <t>sleeve_head_insert_r</t>
+  </si>
+  <si>
+    <t>magnet_ring_insert_part_axial_flat_cut</t>
+  </si>
+  <si>
+    <t>magnet_ring_insert_pos</t>
+  </si>
+  <si>
+    <t>casing_radial_stator_insert_pos</t>
+  </si>
+  <si>
+    <t>stator_radial_screw_d</t>
+  </si>
+  <si>
+    <t>stator_radial_screw_pos</t>
+  </si>
+  <si>
+    <t>rotor_sleeve_in_D</t>
+  </si>
+  <si>
+    <t>rotor_sleeve_out_D</t>
+  </si>
+  <si>
+    <t>rotor_sleeve_h</t>
+  </si>
+  <si>
+    <t>carbon_brush_batt_d</t>
+  </si>
+  <si>
+    <t>carbon_brush_batt_h</t>
   </si>
 </sst>
 </file>
@@ -540,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42.21875" bestFit="1" customWidth="1"/>
@@ -617,431 +731,745 @@
         <v>2</v>
       </c>
       <c r="B9" s="1">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>3</v>
+        <v>93</v>
       </c>
       <c r="B10" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="1">
+        <f>B25</f>
         <v>4</v>
-      </c>
-      <c r="B11" s="1">
-        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B12" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B13" s="1">
-        <v>0.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="1">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B16" s="1">
         <f>B7-B8</f>
         <v>27.5</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B17" s="1">
         <v>3.3</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B18" s="1">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B19" s="1">
         <v>7.1</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B20" s="1">
         <v>3.1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B21" s="1">
         <v>10.3</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B22" s="1">
         <v>1.4</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>77</v>
+      </c>
+      <c r="B23" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="1">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="1">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="B26" s="1">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B27" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B28" s="1">
         <f>B7</f>
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B29" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>74</v>
+      </c>
+      <c r="B30" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" s="1">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>76</v>
+      </c>
+      <c r="B32" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>80</v>
+      </c>
+      <c r="B35" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>81</v>
+      </c>
+      <c r="B36" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>82</v>
+      </c>
+      <c r="B37" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>88</v>
+      </c>
+      <c r="B38" s="1">
         <v>19</v>
       </c>
-      <c r="B24" s="1">
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>92</v>
+      </c>
+      <c r="B39" s="1">
+        <f>14+B25+0.1</f>
+        <v>18.100000000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>19</v>
+      </c>
+      <c r="B40" s="1">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B41" s="1">
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B42" s="1">
         <v>18</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C42" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B43" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B44" s="1">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
         <v>23</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B45" s="1">
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
         <v>24</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B46" s="1">
         <v>1.5</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
         <v>27</v>
       </c>
-      <c r="B31" s="1">
+      <c r="B47" s="1">
         <v>37</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
         <v>25</v>
       </c>
-      <c r="B32" s="1">
+      <c r="B48" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
         <v>26</v>
       </c>
-      <c r="B33" s="1">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
+      <c r="B49" s="1">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
         <v>28</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B50" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
         <v>29</v>
       </c>
-      <c r="B35" s="1">
+      <c r="B51" s="1">
         <f>44</f>
         <v>44</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>30</v>
-      </c>
-      <c r="B36" s="1">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>46</v>
-      </c>
-      <c r="B38" s="1">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>47</v>
-      </c>
-      <c r="B39" s="1">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>48</v>
-      </c>
-      <c r="B40" s="1">
-        <v>7.6</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>49</v>
-      </c>
-      <c r="B41" s="1">
-        <f>B31</f>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>50</v>
-      </c>
-      <c r="B42" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>51</v>
-      </c>
-      <c r="B43" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>52</v>
-      </c>
-      <c r="B44" s="1">
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>55</v>
-      </c>
-      <c r="B45" s="1">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>53</v>
-      </c>
-      <c r="B46" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>54</v>
-      </c>
-      <c r="B47" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>32</v>
-      </c>
-      <c r="B48" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>33</v>
-      </c>
-      <c r="B49" s="1">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>34</v>
-      </c>
-      <c r="B50" s="1">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>35</v>
-      </c>
-      <c r="B51" s="1">
-        <v>2</v>
-      </c>
-    </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B52" s="1">
-        <v>36</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B53" s="1">
-        <v>5.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B54" s="1">
-        <v>7.6</v>
+        <v>36</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B55" s="1">
-        <f>B41</f>
-        <v>37</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B56" s="1">
-        <v>20</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B57" s="1">
-        <v>12</v>
+        <f>B47</f>
+        <v>37</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B58" s="1">
-        <v>5.4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B59" s="1">
-        <v>2.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="B60" s="1">
-        <v>2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
+        <v>55</v>
+      </c>
+      <c r="B61" s="1">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>53</v>
+      </c>
+      <c r="B62" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>54</v>
+      </c>
+      <c r="B63" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>32</v>
+      </c>
+      <c r="B64" s="1">
+        <f>B50</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>33</v>
+      </c>
+      <c r="B65" s="1">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>34</v>
+      </c>
+      <c r="B66" s="1">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>35</v>
+      </c>
+      <c r="B67" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>36</v>
+      </c>
+      <c r="B68" s="1">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>37</v>
+      </c>
+      <c r="B69" s="1">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>38</v>
+      </c>
+      <c r="B70" s="1">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>39</v>
+      </c>
+      <c r="B71" s="1">
+        <f>B57</f>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>56</v>
+      </c>
+      <c r="B72" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>57</v>
+      </c>
+      <c r="B73" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>58</v>
+      </c>
+      <c r="B74" s="1">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>59</v>
+      </c>
+      <c r="B75" s="1">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>60</v>
+      </c>
+      <c r="B76" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
         <v>61</v>
       </c>
-      <c r="B61" s="1">
+      <c r="B77" s="1">
         <v>0.5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>67</v>
+      </c>
+      <c r="B78" s="1">
+        <f>B84-(B85*2)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>68</v>
+      </c>
+      <c r="B79" s="1">
+        <f>B64</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>64</v>
+      </c>
+      <c r="B80" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>69</v>
+      </c>
+      <c r="B81" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>70</v>
+      </c>
+      <c r="B82" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>71</v>
+      </c>
+      <c r="B83" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>62</v>
+      </c>
+      <c r="B84" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>63</v>
+      </c>
+      <c r="B85" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>65</v>
+      </c>
+      <c r="B86" s="1">
+        <v>55</v>
+      </c>
+      <c r="C86" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>66</v>
+      </c>
+      <c r="B87" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>72</v>
+      </c>
+      <c r="B88" s="1">
+        <f>B83</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>83</v>
+      </c>
+      <c r="B89" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>84</v>
+      </c>
+      <c r="B90" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>87</v>
+      </c>
+      <c r="B91" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>85</v>
+      </c>
+      <c r="B92" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>86</v>
+      </c>
+      <c r="B93" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>89</v>
+      </c>
+      <c r="B94" s="1">
+        <f>B38</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>95</v>
+      </c>
+      <c r="B95" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>96</v>
+      </c>
+      <c r="B96" s="1">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>97</v>
+      </c>
+      <c r="B97" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>98</v>
+      </c>
+      <c r="B98" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>99</v>
+      </c>
+      <c r="B99" s="1">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
almost Rev 1.0, full 3d print files
</commit_message>
<xml_diff>
--- a/model/param.xlsx
+++ b/model/param.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zzapa\Desktop\Projekty\elektronika\engine-project\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B44FD8-6B97-49A7-80CF-CDAD2FCA0469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA772FE9-10A8-466A-A7E8-F9A3C2A6DFDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="158">
   <si>
     <t>stator_out_d</t>
   </si>
@@ -336,6 +336,180 @@
   </si>
   <si>
     <t>carbon_brush_batt_h</t>
+  </si>
+  <si>
+    <t>brush_cart_outer_holder_length</t>
+  </si>
+  <si>
+    <t>brush_cart_outer_holder_width</t>
+  </si>
+  <si>
+    <t>brush_cart_outer_holder_arc_r</t>
+  </si>
+  <si>
+    <t>brush_cart_outer_holder_depth</t>
+  </si>
+  <si>
+    <t>brush_cart_outer_holder_arc_pos</t>
+  </si>
+  <si>
+    <t>casing_cart_hole_width</t>
+  </si>
+  <si>
+    <t>casing_cart_hole_corner</t>
+  </si>
+  <si>
+    <t>casing_cart_hole_ang</t>
+  </si>
+  <si>
+    <t>brush_holder_batt_length</t>
+  </si>
+  <si>
+    <t>brush_holder_batt_width</t>
+  </si>
+  <si>
+    <t>brush_holder_batt_depth</t>
+  </si>
+  <si>
+    <t>brush_holder_batt_arc_r</t>
+  </si>
+  <si>
+    <t>brush_holder_batt_insert_flat_length</t>
+  </si>
+  <si>
+    <t>brush_holder_batt_insert_flat_depth</t>
+  </si>
+  <si>
+    <t>brush_holder_batt_brush_hole_d</t>
+  </si>
+  <si>
+    <t>brush_holder_batt_brush_hole_h</t>
+  </si>
+  <si>
+    <t>casing_backsleeve_insert_pos</t>
+  </si>
+  <si>
+    <t>casing_cart_hole_pos</t>
+  </si>
+  <si>
+    <t>casing_sleeve_cut_h</t>
+  </si>
+  <si>
+    <t>casing_sleeve_cut_d</t>
+  </si>
+  <si>
+    <t>name_plate_D</t>
+  </si>
+  <si>
+    <t>name_plate_d</t>
+  </si>
+  <si>
+    <t>name_plate_insert_r</t>
+  </si>
+  <si>
+    <t>name_plate_text_d</t>
+  </si>
+  <si>
+    <t>sleeve_bearing_material_lock_r</t>
+  </si>
+  <si>
+    <t>sleeve_bearing_material_lock_h</t>
+  </si>
+  <si>
+    <t>back_sleeve_D</t>
+  </si>
+  <si>
+    <t>back_sleeve_d</t>
+  </si>
+  <si>
+    <t>back_sleeve_h</t>
+  </si>
+  <si>
+    <t>commutator_plastic_back_plate_lock_h</t>
+  </si>
+  <si>
+    <t>commutator_plastic_back_plate_lock_r</t>
+  </si>
+  <si>
+    <t>commutator_plastic_back_plate_hook_in_r</t>
+  </si>
+  <si>
+    <t>commutator_plastic_back_plate_hook_h</t>
+  </si>
+  <si>
+    <t>back_sleeve_bearing_cup_h</t>
+  </si>
+  <si>
+    <t>back_sleeve_bearing_cup_d</t>
+  </si>
+  <si>
+    <t>back_sleeve_bearing_casing_out_d</t>
+  </si>
+  <si>
+    <t>back_sleeve_bearing_casing_out_width</t>
+  </si>
+  <si>
+    <t>sleeve_seger_cut_pos</t>
+  </si>
+  <si>
+    <t>sleeve_seger_cut_h</t>
+  </si>
+  <si>
+    <t>sleeve_seger_cut_d</t>
+  </si>
+  <si>
+    <t>back_sleeve_corner</t>
+  </si>
+  <si>
+    <t>back_sleeve_cable_hole_pos</t>
+  </si>
+  <si>
+    <t>back_sleeve_cable_hole_d</t>
+  </si>
+  <si>
+    <t>back_sleeve_casing_conn_h</t>
+  </si>
+  <si>
+    <t>back_sleeve_casing_conn_a</t>
+  </si>
+  <si>
+    <t>back_sleeve_casing_conn_ang</t>
+  </si>
+  <si>
+    <t>back_sleeve_casing_conn_cut</t>
+  </si>
+  <si>
+    <t>back_sleeve_casing_conn_insert_pos</t>
+  </si>
+  <si>
+    <t>casing_stand_pos</t>
+  </si>
+  <si>
+    <t>casing_stand_width</t>
+  </si>
+  <si>
+    <t>casing_stand_cylinder_h</t>
+  </si>
+  <si>
+    <t>casing_stand_foot_h</t>
+  </si>
+  <si>
+    <t>casing_stand_foot_width</t>
+  </si>
+  <si>
+    <t>casing_stand_pad_a</t>
+  </si>
+  <si>
+    <t>casing_stand_pad_b</t>
+  </si>
+  <si>
+    <t>casing_stand_pad_spacing_x</t>
+  </si>
+  <si>
+    <t>casing_stand_pad_spacing_y</t>
+  </si>
+  <si>
+    <t>stator_r_out_tolerance</t>
   </si>
 </sst>
 </file>
@@ -654,7 +828,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C157"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42.21875" bestFit="1" customWidth="1"/>
@@ -715,761 +889,1241 @@
         <v>1</v>
       </c>
       <c r="B7" s="1">
-        <v>30</v>
+        <v>30.15</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>0</v>
+        <v>157</v>
       </c>
       <c r="B8" s="1">
-        <v>2.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B9" s="1">
-        <v>45</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>2</v>
       </c>
       <c r="B10" s="1">
-        <v>4</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B11" s="1">
-        <f>B25</f>
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>3</v>
+        <v>94</v>
       </c>
       <c r="B12" s="1">
-        <v>7</v>
+        <f>B26</f>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="1">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B15" s="1">
-        <v>0.4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16" s="1">
-        <f>B7-B8</f>
-        <v>27.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B17" s="1">
-        <v>3.3</v>
+        <f>B7-B9</f>
+        <v>26.95</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B18" s="1">
-        <v>36</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B19" s="1">
-        <v>7.1</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B20" s="1">
-        <v>3.1</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B21" s="1">
-        <v>10.3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B22" s="1">
-        <v>1.4</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>77</v>
+        <v>13</v>
       </c>
       <c r="B23" s="1">
-        <v>8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="B24" s="1">
-        <v>0.17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B25" s="1">
-        <v>4</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>14</v>
+        <v>91</v>
       </c>
       <c r="B26" s="1">
-        <v>80</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B27" s="1">
-        <v>3</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B28" s="1">
-        <f>B7</f>
-        <v>30</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>73</v>
+        <v>16</v>
       </c>
       <c r="B29" s="1">
-        <v>14</v>
+        <f>B7</f>
+        <v>30.15</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B30" s="1">
-        <v>8</v>
+        <v>14.25</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B31" s="1">
-        <v>23</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B32" s="1">
-        <v>6</v>
+        <v>23</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B33" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B34" s="1">
-        <v>20</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B35" s="1">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B36" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B37" s="1">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B38" s="1">
-        <v>19</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B39" s="1">
-        <f>14+B25+0.1</f>
-        <v>18.100000000000001</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="B40" s="1">
-        <v>23</v>
+        <f>14+B26+0.1</f>
+        <v>18.100000000000001</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>18</v>
+        <v>107</v>
       </c>
       <c r="B41" s="1">
-        <v>17</v>
+        <v>90</v>
+      </c>
+      <c r="C41" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="B42" s="1">
-        <v>18</v>
-      </c>
-      <c r="C42" t="s">
-        <v>21</v>
+        <f>B4</f>
+        <v>2.6</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>17</v>
+        <v>106</v>
       </c>
       <c r="B43" s="1">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>22</v>
+        <v>117</v>
       </c>
       <c r="B44" s="1">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>23</v>
+        <v>119</v>
       </c>
       <c r="B45" s="1">
-        <v>32</v>
+        <f>23*2</f>
+        <v>46</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>24</v>
+        <v>118</v>
       </c>
       <c r="B46" s="1">
-        <v>1.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>27</v>
+        <v>116</v>
       </c>
       <c r="B47" s="1">
-        <v>37</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
+        <v>148</v>
+      </c>
+      <c r="B48" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>149</v>
+      </c>
+      <c r="B49" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>150</v>
+      </c>
+      <c r="B50" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>151</v>
+      </c>
+      <c r="B51" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>152</v>
+      </c>
+      <c r="B52" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>153</v>
+      </c>
+      <c r="B53" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>154</v>
+      </c>
+      <c r="B54" s="1">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>155</v>
+      </c>
+      <c r="B55" s="1">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>156</v>
+      </c>
+      <c r="B56" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>19</v>
+      </c>
+      <c r="B57" s="1">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>18</v>
+      </c>
+      <c r="B58" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" s="1">
+        <v>18</v>
+      </c>
+      <c r="C59" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>17</v>
+      </c>
+      <c r="B60" s="1">
+        <f>15-0.03</f>
+        <v>14.97</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>22</v>
+      </c>
+      <c r="B61" s="1">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>23</v>
+      </c>
+      <c r="B62" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>24</v>
+      </c>
+      <c r="B63" s="1">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>27</v>
+      </c>
+      <c r="B64" s="1">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
         <v>25</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B65" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
         <v>26</v>
       </c>
-      <c r="B49" s="1">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
+      <c r="B66" s="1">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
         <v>28</v>
       </c>
-      <c r="B50" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
+      <c r="B67" s="1">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
         <v>29</v>
       </c>
-      <c r="B51" s="1">
+      <c r="B68" s="1">
         <f>44</f>
         <v>44</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>30</v>
-      </c>
-      <c r="B52" s="1">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>31</v>
-      </c>
-      <c r="B53" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>46</v>
-      </c>
-      <c r="B54" s="1">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>47</v>
-      </c>
-      <c r="B55" s="1">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>48</v>
-      </c>
-      <c r="B56" s="1">
-        <v>7.6</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>49</v>
-      </c>
-      <c r="B57" s="1">
-        <f>B47</f>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>50</v>
-      </c>
-      <c r="B58" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>51</v>
-      </c>
-      <c r="B59" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>52</v>
-      </c>
-      <c r="B60" s="1">
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>55</v>
-      </c>
-      <c r="B61" s="1">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>53</v>
-      </c>
-      <c r="B62" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>54</v>
-      </c>
-      <c r="B63" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>32</v>
-      </c>
-      <c r="B64" s="1">
-        <f>B50</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>33</v>
-      </c>
-      <c r="B65" s="1">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>34</v>
-      </c>
-      <c r="B66" s="1">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
-        <v>35</v>
-      </c>
-      <c r="B67" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
-        <v>36</v>
-      </c>
-      <c r="B68" s="1">
-        <v>36</v>
-      </c>
-    </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B69" s="1">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B70" s="1">
-        <v>7.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B71" s="1">
-        <f>B57</f>
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B72" s="1">
-        <v>20</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="B73" s="1">
-        <v>12</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B74" s="1">
-        <v>5.4</v>
+        <f>B64</f>
+        <v>37</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="B75" s="1">
-        <v>2.5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B76" s="1">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="B77" s="1">
-        <v>0.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="B78" s="1">
-        <f>B84-(B85*2)</f>
-        <v>20</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B79" s="1">
-        <f>B64</f>
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
+        <v>54</v>
+      </c>
+      <c r="B80" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>32</v>
+      </c>
+      <c r="B81" s="1">
+        <f>B67</f>
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>33</v>
+      </c>
+      <c r="B82" s="1">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>34</v>
+      </c>
+      <c r="B83" s="1">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>35</v>
+      </c>
+      <c r="B84" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>36</v>
+      </c>
+      <c r="B85" s="1">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>37</v>
+      </c>
+      <c r="B86" s="1">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>38</v>
+      </c>
+      <c r="B87" s="1">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>39</v>
+      </c>
+      <c r="B88" s="1">
+        <f>B74</f>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>56</v>
+      </c>
+      <c r="B89" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>57</v>
+      </c>
+      <c r="B90" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>58</v>
+      </c>
+      <c r="B91" s="1">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>59</v>
+      </c>
+      <c r="B92" s="1">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>60</v>
+      </c>
+      <c r="B93" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>61</v>
+      </c>
+      <c r="B94" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>67</v>
+      </c>
+      <c r="B95" s="1">
+        <f>B105-(B106*2)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>68</v>
+      </c>
+      <c r="B96" s="1">
+        <f>B81</f>
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
         <v>64</v>
       </c>
-      <c r="B80" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
+      <c r="B97" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
         <v>69</v>
       </c>
-      <c r="B81" s="1">
+      <c r="B98" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>70</v>
+      </c>
+      <c r="B99" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>71</v>
+      </c>
+      <c r="B100" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
-        <v>70</v>
-      </c>
-      <c r="B82" s="1">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102" s="1">
+        <f>23.8/2</f>
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103" s="1">
+        <v>11.15</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>62</v>
+      </c>
+      <c r="B105" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>63</v>
+      </c>
+      <c r="B106" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>65</v>
+      </c>
+      <c r="B107" s="1">
+        <v>55</v>
+      </c>
+      <c r="C107" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>66</v>
+      </c>
+      <c r="B108" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>72</v>
+      </c>
+      <c r="B109" s="1">
+        <f>B100</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>83</v>
+      </c>
+      <c r="B110" s="1">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>84</v>
+      </c>
+      <c r="B111" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>87</v>
+      </c>
+      <c r="B112" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>85</v>
+      </c>
+      <c r="B113" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>86</v>
+      </c>
+      <c r="B114" s="1">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>89</v>
+      </c>
+      <c r="B115" s="1">
+        <f>B39</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>124</v>
+      </c>
+      <c r="B116" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
+        <v>125</v>
+      </c>
+      <c r="B117" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
+        <v>137</v>
+      </c>
+      <c r="B118" s="1">
+        <v>7.15</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>138</v>
+      </c>
+      <c r="B119" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>139</v>
+      </c>
+      <c r="B120" s="1">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>95</v>
+      </c>
+      <c r="B121" s="1">
+        <f>B96+0.05</f>
+        <v>8.15</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>96</v>
+      </c>
+      <c r="B122" s="1">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>97</v>
+      </c>
+      <c r="B123" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>98</v>
+      </c>
+      <c r="B124" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>99</v>
+      </c>
+      <c r="B125" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>100</v>
+      </c>
+      <c r="B126" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>101</v>
+      </c>
+      <c r="B127" s="1">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
+        <v>103</v>
+      </c>
+      <c r="B128" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A129" t="s">
+        <v>102</v>
+      </c>
+      <c r="B129" s="1">
+        <f>B29+B28</f>
+        <v>33.15</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>104</v>
+      </c>
+      <c r="B130" s="1">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A131" t="s">
+        <v>108</v>
+      </c>
+      <c r="B131" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
+        <v>109</v>
+      </c>
+      <c r="B132" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>110</v>
+      </c>
+      <c r="B133" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>111</v>
+      </c>
+      <c r="B134" s="1">
+        <f>B29</f>
+        <v>30.15</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>112</v>
+      </c>
+      <c r="B135" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
-        <v>71</v>
-      </c>
-      <c r="B83" s="1">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>113</v>
+      </c>
+      <c r="B136" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>114</v>
+      </c>
+      <c r="B137" s="1">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>115</v>
+      </c>
+      <c r="B138" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>120</v>
+      </c>
+      <c r="B139" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>121</v>
+      </c>
+      <c r="B140" s="1">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>122</v>
+      </c>
+      <c r="B141" s="1">
+        <f>B115</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>123</v>
+      </c>
+      <c r="B142" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>126</v>
+      </c>
+      <c r="B143" s="1">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>127</v>
+      </c>
+      <c r="B144" s="1">
+        <f>B110*2</f>
+        <v>22.2</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>128</v>
+      </c>
+      <c r="B145" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>140</v>
+      </c>
+      <c r="B146" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>133</v>
+      </c>
+      <c r="B147" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A148" t="s">
+        <v>134</v>
+      </c>
+      <c r="B148" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>135</v>
+      </c>
+      <c r="B149" s="1">
+        <f>60-0.2</f>
+        <v>59.8</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>136</v>
+      </c>
+      <c r="B150" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
+        <v>141</v>
+      </c>
+      <c r="B151" s="1">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>142</v>
+      </c>
+      <c r="B152" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>143</v>
+      </c>
+      <c r="B153" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>144</v>
+      </c>
+      <c r="B154" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>62</v>
-      </c>
-      <c r="B84" s="1">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>63</v>
-      </c>
-      <c r="B85" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A86" t="s">
-        <v>65</v>
-      </c>
-      <c r="B86" s="1">
-        <v>55</v>
-      </c>
-      <c r="C86" t="s">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>145</v>
+      </c>
+      <c r="B155" s="1">
+        <v>20</v>
+      </c>
+      <c r="C155" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
-        <v>66</v>
-      </c>
-      <c r="B87" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
-        <v>72</v>
-      </c>
-      <c r="B88" s="1">
-        <f>B83</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A89" t="s">
-        <v>83</v>
-      </c>
-      <c r="B89" s="1">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A90" t="s">
-        <v>84</v>
-      </c>
-      <c r="B90" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
-        <v>87</v>
-      </c>
-      <c r="B91" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A92" t="s">
-        <v>85</v>
-      </c>
-      <c r="B92" s="1">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
-        <v>86</v>
-      </c>
-      <c r="B93" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
-        <v>89</v>
-      </c>
-      <c r="B94" s="1">
-        <f>B38</f>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
-        <v>95</v>
-      </c>
-      <c r="B95" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
-        <v>96</v>
-      </c>
-      <c r="B96" s="1">
-        <v>10.5</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
-        <v>97</v>
-      </c>
-      <c r="B97" s="1">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
-        <v>98</v>
-      </c>
-      <c r="B98" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A99" t="s">
-        <v>99</v>
-      </c>
-      <c r="B99" s="1">
-        <v>10</v>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>146</v>
+      </c>
+      <c r="B156" s="1">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>147</v>
+      </c>
+      <c r="B157" s="1">
+        <v>4.9000000000000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Full inventor assembly v1.0
</commit_message>
<xml_diff>
--- a/model/param.xlsx
+++ b/model/param.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zzapa\Desktop\Projekty\elektronika\engine-project\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA772FE9-10A8-466A-A7E8-F9A3C2A6DFDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9BE15E-4388-41CE-835B-95A736C00A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="160">
   <si>
     <t>stator_out_d</t>
   </si>
@@ -510,6 +510,12 @@
   </si>
   <si>
     <t>stator_r_out_tolerance</t>
+  </si>
+  <si>
+    <t>shaft_D_h</t>
+  </si>
+  <si>
+    <t>shaft_D_size</t>
   </si>
 </sst>
 </file>
@@ -828,7 +834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C157"/>
+  <dimension ref="A1:C159"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42.21875" bestFit="1" customWidth="1"/>
@@ -1379,326 +1385,326 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>28</v>
+        <v>158</v>
       </c>
       <c r="B67" s="1">
-        <v>8.1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
+        <v>159</v>
+      </c>
+      <c r="B68" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>28</v>
+      </c>
+      <c r="B69" s="1">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
         <v>29</v>
       </c>
-      <c r="B68" s="1">
+      <c r="B70" s="1">
         <f>44</f>
         <v>44</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>30</v>
-      </c>
-      <c r="B69" s="1">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>31</v>
-      </c>
-      <c r="B70" s="1">
-        <v>2</v>
-      </c>
-    </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="B71" s="1">
-        <v>36</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="B72" s="1">
-        <v>5.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B73" s="1">
-        <v>7.6</v>
+        <v>36</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
+        <v>47</v>
+      </c>
+      <c r="B74" s="1">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>48</v>
+      </c>
+      <c r="B75" s="1">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
         <v>49</v>
       </c>
-      <c r="B74" s="1">
+      <c r="B76" s="1">
         <f>B64</f>
         <v>37</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
-        <v>50</v>
-      </c>
-      <c r="B75" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>51</v>
-      </c>
-      <c r="B76" s="1">
-        <v>12</v>
-      </c>
-    </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B77" s="1">
-        <v>5.4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B78" s="1">
-        <v>2.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B79" s="1">
-        <v>2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B80" s="1">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="B81" s="1">
-        <f>B67</f>
-        <v>8.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="B82" s="1">
-        <v>44</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B83" s="1">
-        <v>3.5</v>
+        <f>B69</f>
+        <v>8.1</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B84" s="1">
-        <v>2</v>
+        <v>44</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B85" s="1">
-        <v>36</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B86" s="1">
-        <v>5.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B87" s="1">
-        <v>7.6</v>
+        <v>36</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B88" s="1">
-        <f>B74</f>
-        <v>37</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="B89" s="1">
-        <v>20</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="B90" s="1">
-        <v>12</v>
+        <f>B76</f>
+        <v>37</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B91" s="1">
-        <v>5.4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B92" s="1">
-        <v>2.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B93" s="1">
-        <v>2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B94" s="1">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B95" s="1">
-        <f>B105-(B106*2)</f>
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B96" s="1">
-        <f>B81</f>
-        <v>8.1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B97" s="1">
-        <v>17</v>
+        <f>B107-(B108*2)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B98" s="1">
-        <v>0.5</v>
+        <f>B83</f>
+        <v>8.1</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B99" s="1">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B100" s="1">
-        <v>3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>129</v>
+        <v>70</v>
       </c>
       <c r="B101" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
+        <v>71</v>
+      </c>
+      <c r="B102" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>129</v>
+      </c>
+      <c r="B103" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
         <v>130</v>
       </c>
-      <c r="B102" s="1">
+      <c r="B104" s="1">
         <f>23.8/2</f>
         <v>11.9</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
-        <v>131</v>
-      </c>
-      <c r="B103" s="1">
-        <v>11.15</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
-        <v>132</v>
-      </c>
-      <c r="B104" s="1">
-        <v>1</v>
-      </c>
-    </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>62</v>
+        <v>131</v>
       </c>
       <c r="B105" s="1">
-        <v>22</v>
+        <v>11.15</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>63</v>
+        <v>132</v>
       </c>
       <c r="B106" s="1">
         <v>1</v>
@@ -1706,181 +1712,181 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B107" s="1">
-        <v>55</v>
-      </c>
-      <c r="C107" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B108" s="1">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B109" s="1">
-        <f>B100</f>
-        <v>3</v>
+        <v>55</v>
+      </c>
+      <c r="C109" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="B110" s="1">
-        <v>11.1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="B111" s="1">
+        <f>B102</f>
         <v>3</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B112" s="1">
-        <v>7</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B113" s="1">
-        <v>22</v>
+        <v>3</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B114" s="1">
-        <v>4.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
+        <v>85</v>
+      </c>
+      <c r="B115" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>86</v>
+      </c>
+      <c r="B116" s="1">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
         <v>89</v>
       </c>
-      <c r="B115" s="1">
+      <c r="B117" s="1">
         <f>B39</f>
         <v>19</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
-        <v>124</v>
-      </c>
-      <c r="B116" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A117" t="s">
-        <v>125</v>
-      </c>
-      <c r="B117" s="1">
-        <v>2</v>
-      </c>
-    </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="B118" s="1">
-        <v>7.15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="B119" s="1">
-        <v>1.1000000000000001</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B120" s="1">
-        <v>23</v>
+        <v>7.15</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>95</v>
+        <v>138</v>
       </c>
       <c r="B121" s="1">
-        <f>B96+0.05</f>
-        <v>8.15</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="B122" s="1">
-        <v>10.5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B123" s="1">
-        <v>32</v>
+        <f>B98+0.05</f>
+        <v>8.15</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B124" s="1">
-        <v>4</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B125" s="1">
-        <v>8</v>
+        <v>32</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B126" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B127" s="1">
-        <v>5.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B128" s="1">
         <v>10</v>
@@ -1888,40 +1894,40 @@
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
+        <v>101</v>
+      </c>
+      <c r="B129" s="1">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>103</v>
+      </c>
+      <c r="B130" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A131" t="s">
         <v>102</v>
       </c>
-      <c r="B129" s="1">
+      <c r="B131" s="1">
         <f>B29+B28</f>
         <v>33.15</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A130" t="s">
-        <v>104</v>
-      </c>
-      <c r="B130" s="1">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A131" t="s">
-        <v>108</v>
-      </c>
-      <c r="B131" s="1">
-        <v>10</v>
-      </c>
-    </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B132" s="1">
-        <v>16</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B133" s="1">
         <v>10</v>
@@ -1929,200 +1935,216 @@
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
+        <v>109</v>
+      </c>
+      <c r="B134" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>110</v>
+      </c>
+      <c r="B135" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
         <v>111</v>
       </c>
-      <c r="B134" s="1">
+      <c r="B136" s="1">
         <f>B29</f>
         <v>30.15</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A135" t="s">
-        <v>112</v>
-      </c>
-      <c r="B135" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A136" t="s">
-        <v>113</v>
-      </c>
-      <c r="B136" s="1">
-        <v>6</v>
-      </c>
-    </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B137" s="1">
-        <v>4.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B138" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B139" s="1">
-        <v>45</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B140" s="1">
-        <v>28</v>
+        <v>10</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B141" s="1">
-        <f>B115</f>
-        <v>19</v>
+        <v>45</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B142" s="1">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B143" s="1">
-        <v>66</v>
+        <f>B117</f>
+        <v>19</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B144" s="1">
-        <f>B110*2</f>
-        <v>22.2</v>
+        <v>40</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B145" s="1">
-        <v>5</v>
+        <v>66</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="B146" s="1">
-        <v>1</v>
+        <f>B112*2</f>
+        <v>22.2</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B147" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B148" s="1">
-        <v>26</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
+        <v>133</v>
+      </c>
+      <c r="B149" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>134</v>
+      </c>
+      <c r="B150" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
         <v>135</v>
       </c>
-      <c r="B149" s="1">
+      <c r="B151" s="1">
         <f>60-0.2</f>
         <v>59.8</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A150" t="s">
-        <v>136</v>
-      </c>
-      <c r="B150" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A151" t="s">
-        <v>141</v>
-      </c>
-      <c r="B151" s="1">
-        <v>21</v>
-      </c>
-    </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="B152" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B153" s="1">
-        <v>9</v>
+        <v>21</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B154" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B155" s="1">
-        <v>20</v>
-      </c>
-      <c r="C155" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B156" s="1">
-        <v>0.2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
+        <v>145</v>
+      </c>
+      <c r="B157" s="1">
+        <v>20</v>
+      </c>
+      <c r="C157" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>146</v>
+      </c>
+      <c r="B158" s="1">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
         <v>147</v>
       </c>
-      <c r="B157" s="1">
+      <c r="B159" s="1">
         <v>4.9000000000000004</v>
       </c>
     </row>

</xml_diff>